<commit_message>
modify map-handelrs.js to try to modify zoom in phones / added new data for SNMV
</commit_message>
<xml_diff>
--- a/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvHomiEdad.xlsx
+++ b/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvHomiEdad.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Sistema_de_Notificacion_de_Muertes_Violentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9DA98E-F36D-4B5A-8647-5F3F94C495C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243C116E-3FB6-4B59-A8B9-A73DE0346859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4008" yWindow="1368" windowWidth="17280" windowHeight="9420" xr2:uid="{158DB65A-6E55-0941-A295-AA375E07226E}"/>
+    <workbookView xWindow="3660" yWindow="2124" windowWidth="11424" windowHeight="9420" xr2:uid="{158DB65A-6E55-0941-A295-AA375E07226E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -145,7 +145,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -544,6 +544,7 @@
         <v>1</v>
       </c>
       <c r="L2" s="5">
+        <f>SUM(B2:K2)</f>
         <v>23</v>
       </c>
     </row>
@@ -582,6 +583,7 @@
         <v>9</v>
       </c>
       <c r="L3" s="5">
+        <f t="shared" ref="L3:L7" si="0">SUM(B3:K3)</f>
         <v>211</v>
       </c>
     </row>
@@ -617,10 +619,11 @@
         <v>22</v>
       </c>
       <c r="K4" s="3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L4" s="5">
-        <v>250</v>
+        <f t="shared" si="0"/>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -634,7 +637,7 @@
         <v>27</v>
       </c>
       <c r="D5" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="3">
         <v>16</v>
@@ -658,7 +661,8 @@
         <v>7</v>
       </c>
       <c r="L5" s="5">
-        <v>209</v>
+        <f>SUM(B5:K5)</f>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -693,10 +697,11 @@
         <v>24</v>
       </c>
       <c r="K6" s="5">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L6" s="5">
-        <v>161</v>
+        <f t="shared" si="0"/>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -734,6 +739,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="5">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
@@ -741,38 +747,49 @@
       <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="5">
+        <f t="shared" ref="B8:J8" si="1">SUM(B2:B7)</f>
         <v>90</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="5">
+        <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="D8" s="3">
-        <v>97</v>
-      </c>
-      <c r="E8" s="3">
+      <c r="D8" s="5">
+        <f t="shared" si="1"/>
+        <v>98</v>
+      </c>
+      <c r="E8" s="5">
+        <f t="shared" si="1"/>
         <v>86</v>
       </c>
       <c r="F8" s="5">
+        <f t="shared" si="1"/>
         <v>69</v>
       </c>
       <c r="G8" s="5">
+        <f t="shared" si="1"/>
         <v>84</v>
       </c>
       <c r="H8" s="5">
+        <f t="shared" si="1"/>
         <v>92</v>
       </c>
       <c r="I8" s="5">
+        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="J8" s="5">
+        <f t="shared" si="1"/>
         <v>91</v>
       </c>
       <c r="K8" s="5">
-        <v>51</v>
+        <f>SUM(K2:K7)</f>
+        <v>54</v>
       </c>
       <c r="L8" s="5">
-        <v>857</v>
+        <f>SUM(L2:L7)</f>
+        <v>861</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -784,7 +801,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -793,7 +810,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -802,7 +819,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -811,7 +828,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -820,7 +837,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>

</xml_diff>